<commit_message>
fix(epirank): realign Flu and NV tables to ISO 2015-2019 (261 weeks)
- rename Flu.xlsx -> flu.xlsx and drop 2020 from both flu and nv: sheet names now 2015_2019, flu window = x731..x991 (261 weeks) instead of trailing 312 columns, nv years = 2015-2019
- build_tables.py: derive the flu week window from calendar dates (FLU_X1=2001-01-01 anchor) instead of a hardcoded column count; drop NV_POP_FALLBACK
- update EpiRank_GUI (原_Germany / 改_Germany) file lists and log messages for flu.xlsx
- out.py: compare EpiRank_原 vs EpiRank_改 instead of the Germany folders
- refresh ERA results and 数据说明.md accordingly
</commit_message>
<xml_diff>
--- a/EpiRank_原/ERA_result_d_0.95_daytime_0.5_loops_309.xlsx
+++ b/EpiRank_原/ERA_result_d_0.95_daytime_0.5_loops_309.xlsx
@@ -1179,10 +1179,10 @@
         <v>0.01205</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z5" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA5" s="3" t="n">
         <v>11</v>
@@ -1334,7 +1334,7 @@
         <v>0.006652</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z6" s="3" t="n">
         <v>0</v>
@@ -2708,10 +2708,10 @@
         <v>0.004698</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z15" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA15" s="3" t="n">
         <v>4</v>
@@ -3008,10 +3008,10 @@
         <v>0.008274999999999999</v>
       </c>
       <c r="Y17" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA17" s="3" t="n">
         <v>4</v>
@@ -3158,10 +3158,10 @@
         <v>0.008586</v>
       </c>
       <c r="Y18" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>3</v>
@@ -3308,10 +3308,10 @@
         <v>0.011024</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="3" t="n">
         <v>8</v>
@@ -4268,10 +4268,10 @@
         <v>0.007023</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z26" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA26" s="3" t="n">
         <v>8</v>
@@ -4918,10 +4918,10 @@
         <v>0.004713</v>
       </c>
       <c r="Y31" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z31" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA31" s="3" t="n">
         <v>7</v>
@@ -5038,10 +5038,10 @@
         <v>0.005408</v>
       </c>
       <c r="Y32" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z32" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA32" s="3" t="n">
         <v>7</v>
@@ -5521,7 +5521,7 @@
         <v>0</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA36" s="3" t="n">
         <v>5</v>
@@ -6718,10 +6718,10 @@
         <v>0.007706</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z46" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA46" s="3" t="n">
         <v>2</v>
@@ -6958,10 +6958,10 @@
         <v>0.006948</v>
       </c>
       <c r="Y48" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z48" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA48" s="3" t="n">
         <v>3</v>
@@ -7201,7 +7201,7 @@
         <v>0</v>
       </c>
       <c r="Z50" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA50" s="3" t="n">
         <v>5</v>
@@ -7438,7 +7438,7 @@
         <v>0.005555</v>
       </c>
       <c r="Y52" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z52" s="3" t="n">
         <v>-0</v>
@@ -7678,10 +7678,10 @@
         <v>0.004587</v>
       </c>
       <c r="Y54" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z54" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA54" s="3" t="n">
         <v>2</v>
@@ -8398,7 +8398,7 @@
         <v>0.004618</v>
       </c>
       <c r="Y60" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z60" s="3" t="n">
         <v>-0</v>
@@ -8878,7 +8878,7 @@
         <v>0.0015</v>
       </c>
       <c r="Y64" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z64" s="3" t="n">
         <v>-0</v>
@@ -9578,10 +9578,10 @@
         <v>0.006096</v>
       </c>
       <c r="Y70" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z70" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA70" s="3" t="n">
         <v>1</v>
@@ -10241,7 +10241,7 @@
         <v>-0</v>
       </c>
       <c r="Z76" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA76" s="3" t="n">
         <v>0</v>
@@ -10348,10 +10348,10 @@
         <v>0.002616</v>
       </c>
       <c r="Y77" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z77" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA77" s="3" t="n">
         <v>2</v>
@@ -10458,10 +10458,10 @@
         <v>0.002491</v>
       </c>
       <c r="Y78" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z78" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA78" s="3" t="n">
         <v>6</v>
@@ -10681,7 +10681,7 @@
         <v>0</v>
       </c>
       <c r="Z80" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA80" s="3" t="n">
         <v>4</v>
@@ -11338,7 +11338,7 @@
         <v>0.003041</v>
       </c>
       <c r="Y86" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z86" s="3" t="n">
         <v>-0</v>
@@ -11558,10 +11558,10 @@
         <v>0.002613</v>
       </c>
       <c r="Y88" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z88" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA88" s="3" t="n">
         <v>2</v>
@@ -11998,10 +11998,10 @@
         <v>0.003408</v>
       </c>
       <c r="Y92" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z92" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA92" s="3" t="n">
         <v>1</v>
@@ -12108,10 +12108,10 @@
         <v>0.003716</v>
       </c>
       <c r="Y93" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z93" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA93" s="3" t="n">
         <v>0</v>
@@ -12328,10 +12328,10 @@
         <v>0.002268</v>
       </c>
       <c r="Y95" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z95" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA95" s="3" t="n">
         <v>0</v>
@@ -12768,10 +12768,10 @@
         <v>0.003882</v>
       </c>
       <c r="Y99" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z99" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA99" s="3" t="n">
         <v>0</v>
@@ -12878,10 +12878,10 @@
         <v>0.003369</v>
       </c>
       <c r="Y100" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z100" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA100" s="3" t="n">
         <v>2</v>
@@ -13868,10 +13868,10 @@
         <v>0.002802</v>
       </c>
       <c r="Y109" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z109" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA109" s="3" t="n">
         <v>0</v>
@@ -14091,7 +14091,7 @@
         <v>0</v>
       </c>
       <c r="Z111" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA111" s="3" t="n">
         <v>2</v>
@@ -14858,10 +14858,10 @@
         <v>0.002496</v>
       </c>
       <c r="Y118" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z118" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA118" s="3" t="n">
         <v>1</v>
@@ -15521,7 +15521,7 @@
         <v>0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>0</v>
@@ -15628,10 +15628,10 @@
         <v>0.002787</v>
       </c>
       <c r="Y125" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>2</v>
@@ -15741,7 +15741,7 @@
         <v>0</v>
       </c>
       <c r="Z126" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA126" s="3" t="n">
         <v>0</v>
@@ -15848,10 +15848,10 @@
         <v>0.002579</v>
       </c>
       <c r="Y127" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z127" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA127" s="3" t="n">
         <v>0</v>
@@ -16068,10 +16068,10 @@
         <v>0.002014</v>
       </c>
       <c r="Y129" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z129" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA129" s="3" t="n">
         <v>3</v>
@@ -16288,10 +16288,10 @@
         <v>0.00191</v>
       </c>
       <c r="Y131" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z131" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA131" s="3" t="n">
         <v>1</v>
@@ -16508,10 +16508,10 @@
         <v>0.003344</v>
       </c>
       <c r="Y133" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z133" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA133" s="3" t="n">
         <v>3</v>
@@ -16728,10 +16728,10 @@
         <v>0.004587</v>
       </c>
       <c r="Y135" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z135" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA135" s="3" t="n">
         <v>0</v>
@@ -16838,10 +16838,10 @@
         <v>0.002116</v>
       </c>
       <c r="Y136" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z136" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA136" s="3" t="n">
         <v>0</v>
@@ -17058,10 +17058,10 @@
         <v>0.002491</v>
       </c>
       <c r="Y138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA138" s="3" t="n">
         <v>2</v>
@@ -17388,7 +17388,7 @@
         <v>0.001759</v>
       </c>
       <c r="Y141" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z141" s="3" t="n">
         <v>-0</v>
@@ -17718,10 +17718,10 @@
         <v>0.005244</v>
       </c>
       <c r="Y144" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z144" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA144" s="3" t="n">
         <v>2</v>
@@ -18488,10 +18488,10 @@
         <v>0.002174</v>
       </c>
       <c r="Y151" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z151" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA151" s="3" t="n">
         <v>1</v>
@@ -18711,7 +18711,7 @@
         <v>0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>0</v>
@@ -18818,10 +18818,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y154" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z154" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA154" s="3" t="n">
         <v>0</v>
@@ -19258,10 +19258,10 @@
         <v>0.003403</v>
       </c>
       <c r="Y158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>0</v>
@@ -19478,10 +19478,10 @@
         <v>0.004473</v>
       </c>
       <c r="Y160" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z160" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA160" s="3" t="n">
         <v>1</v>
@@ -19808,10 +19808,10 @@
         <v>0.002964</v>
       </c>
       <c r="Y163" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z163" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA163" s="3" t="n">
         <v>3</v>
@@ -20028,10 +20028,10 @@
         <v>0.002813</v>
       </c>
       <c r="Y165" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z165" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA165" s="3" t="n">
         <v>1</v>
@@ -20141,7 +20141,7 @@
         <v>0</v>
       </c>
       <c r="Z166" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA166" s="3" t="n">
         <v>2</v>
@@ -20248,10 +20248,10 @@
         <v>0.002432</v>
       </c>
       <c r="Y167" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z167" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA167" s="3" t="n">
         <v>1</v>
@@ -20468,10 +20468,10 @@
         <v>0.001501</v>
       </c>
       <c r="Y169" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z169" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA169" s="3" t="n">
         <v>1</v>
@@ -20908,10 +20908,10 @@
         <v>0.003364</v>
       </c>
       <c r="Y173" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z173" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA173" s="3" t="n">
         <v>0</v>
@@ -21241,7 +21241,7 @@
         <v>0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>1</v>
@@ -21461,7 +21461,7 @@
         <v>0</v>
       </c>
       <c r="Z178" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA178" s="3" t="n">
         <v>2</v>
@@ -21678,10 +21678,10 @@
         <v>0.001235</v>
       </c>
       <c r="Y180" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z180" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA180" s="3" t="n">
         <v>1</v>
@@ -21791,7 +21791,7 @@
         <v>0</v>
       </c>
       <c r="Z181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA181" s="3" t="n">
         <v>0</v>
@@ -21898,10 +21898,10 @@
         <v>0.0011</v>
       </c>
       <c r="Y182" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z182" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA182" s="3" t="n">
         <v>0</v>
@@ -22121,7 +22121,7 @@
         <v>0</v>
       </c>
       <c r="Z184" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA184" s="3" t="n">
         <v>0</v>
@@ -22341,7 +22341,7 @@
         <v>-0</v>
       </c>
       <c r="Z186" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA186" s="3" t="n">
         <v>1</v>
@@ -22448,10 +22448,10 @@
         <v>0.002618</v>
       </c>
       <c r="Y187" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z187" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA187" s="3" t="n">
         <v>0</v>
@@ -22558,10 +22558,10 @@
         <v>0.001669</v>
       </c>
       <c r="Y188" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z188" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA188" s="3" t="n">
         <v>0</v>
@@ -22668,10 +22668,10 @@
         <v>0.0009700000000000001</v>
       </c>
       <c r="Y189" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z189" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA189" s="3" t="n">
         <v>3</v>
@@ -22888,10 +22888,10 @@
         <v>0.001708</v>
       </c>
       <c r="Y191" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z191" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA191" s="3" t="n">
         <v>0</v>
@@ -22998,7 +22998,7 @@
         <v>0.002238</v>
       </c>
       <c r="Y192" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z192" s="3" t="n">
         <v>0</v>
@@ -23551,7 +23551,7 @@
         <v>0</v>
       </c>
       <c r="Z197" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA197" s="3" t="n">
         <v>1</v>
@@ -23878,10 +23878,10 @@
         <v>0.001686</v>
       </c>
       <c r="Y200" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z200" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA200" s="3" t="n">
         <v>1</v>
@@ -23988,7 +23988,7 @@
         <v>0.001259</v>
       </c>
       <c r="Y201" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z201" s="3" t="n">
         <v>-0</v>
@@ -24318,7 +24318,7 @@
         <v>0.002004</v>
       </c>
       <c r="Y204" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z204" s="3" t="n">
         <v>0</v>
@@ -24538,7 +24538,7 @@
         <v>0.001782</v>
       </c>
       <c r="Y206" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z206" s="3" t="n">
         <v>-0</v>
@@ -24978,10 +24978,10 @@
         <v>0.001245</v>
       </c>
       <c r="Y210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>0</v>
@@ -25311,7 +25311,7 @@
         <v>0</v>
       </c>
       <c r="Z213" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA213" s="3" t="n">
         <v>6</v>
@@ -25528,10 +25528,10 @@
         <v>0.002059</v>
       </c>
       <c r="Y215" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z215" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA215" s="3" t="n">
         <v>0</v>
@@ -25638,10 +25638,10 @@
         <v>0.0008140000000000001</v>
       </c>
       <c r="Y216" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z216" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA216" s="3" t="n">
         <v>0</v>
@@ -25751,7 +25751,7 @@
         <v>0</v>
       </c>
       <c r="Z217" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA217" s="3" t="n">
         <v>0</v>
@@ -25861,7 +25861,7 @@
         <v>-0</v>
       </c>
       <c r="Z218" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA218" s="3" t="n">
         <v>0</v>
@@ -26078,10 +26078,10 @@
         <v>0.001943</v>
       </c>
       <c r="Y220" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z220" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA220" s="3" t="n">
         <v>0</v>
@@ -26391,7 +26391,7 @@
         <v>-0</v>
       </c>
       <c r="Z223" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA223" s="3" t="n">
         <v>6</v>
@@ -26588,10 +26588,10 @@
         <v>0.00135</v>
       </c>
       <c r="Y225" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z225" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA225" s="3" t="n">
         <v>0</v>
@@ -26788,10 +26788,10 @@
         <v>0.001152</v>
       </c>
       <c r="Y227" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z227" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA227" s="3" t="n">
         <v>0</v>
@@ -26988,7 +26988,7 @@
         <v>0.00125</v>
       </c>
       <c r="Y229" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z229" s="3" t="n">
         <v>0</v>
@@ -27091,7 +27091,7 @@
         <v>0</v>
       </c>
       <c r="Z230" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA230" s="3" t="n">
         <v>2</v>
@@ -27291,7 +27291,7 @@
         <v>0</v>
       </c>
       <c r="Z232" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA232" s="3" t="n">
         <v>0</v>
@@ -27488,7 +27488,7 @@
         <v>0.001</v>
       </c>
       <c r="Y234" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z234" s="3" t="n">
         <v>-0</v>
@@ -27588,10 +27588,10 @@
         <v>0.001309</v>
       </c>
       <c r="Y235" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z235" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA235" s="3" t="n">
         <v>0</v>
@@ -27688,7 +27688,7 @@
         <v>0.001592</v>
       </c>
       <c r="Y236" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z236" s="3" t="n">
         <v>-0</v>
@@ -27788,10 +27788,10 @@
         <v>0.00164</v>
       </c>
       <c r="Y237" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z237" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA237" s="3" t="n">
         <v>0</v>
@@ -27891,7 +27891,7 @@
         <v>0</v>
       </c>
       <c r="Z238" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA238" s="3" t="n">
         <v>2</v>
@@ -28188,7 +28188,7 @@
         <v>0.001513</v>
       </c>
       <c r="Y241" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z241" s="3" t="n">
         <v>0</v>
@@ -28391,7 +28391,7 @@
         <v>0</v>
       </c>
       <c r="Z243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA243" s="3" t="n">
         <v>0</v>
@@ -28491,7 +28491,7 @@
         <v>0</v>
       </c>
       <c r="Z244" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA244" s="3" t="n">
         <v>3</v>
@@ -28591,7 +28591,7 @@
         <v>0</v>
       </c>
       <c r="Z245" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA245" s="3" t="n">
         <v>1</v>
@@ -28688,7 +28688,7 @@
         <v>0.002084</v>
       </c>
       <c r="Y246" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z246" s="3" t="n">
         <v>-0</v>
@@ -28791,7 +28791,7 @@
         <v>-0</v>
       </c>
       <c r="Z247" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA247" s="3" t="n">
         <v>0</v>
@@ -28988,10 +28988,10 @@
         <v>0.001148</v>
       </c>
       <c r="Y249" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z249" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA249" s="3" t="n">
         <v>0</v>
@@ -29088,10 +29088,10 @@
         <v>0.001877</v>
       </c>
       <c r="Y250" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z250" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA250" s="3" t="n">
         <v>0</v>
@@ -29391,7 +29391,7 @@
         <v>0</v>
       </c>
       <c r="Z253" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA253" s="3" t="n">
         <v>2</v>
@@ -29488,10 +29488,10 @@
         <v>0.001296</v>
       </c>
       <c r="Y254" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z254" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA254" s="3" t="n">
         <v>1</v>
@@ -29691,7 +29691,7 @@
         <v>-0</v>
       </c>
       <c r="Z256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA256" s="3" t="n">
         <v>0</v>
@@ -29991,7 +29991,7 @@
         <v>-0</v>
       </c>
       <c r="Z259" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA259" s="3" t="n">
         <v>0</v>
@@ -30091,7 +30091,7 @@
         <v>0</v>
       </c>
       <c r="Z260" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA260" s="3" t="n">
         <v>0</v>
@@ -30188,7 +30188,7 @@
         <v>0.001556</v>
       </c>
       <c r="Y261" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z261" s="3" t="n">
         <v>-0</v>
@@ -30288,7 +30288,7 @@
         <v>0.000785</v>
       </c>
       <c r="Y262" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z262" s="3" t="n">
         <v>-0</v>
@@ -30588,7 +30588,7 @@
         <v>0.00079</v>
       </c>
       <c r="Y265" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z265" s="3" t="n">
         <v>-0</v>
@@ -30788,7 +30788,7 @@
         <v>0.001386</v>
       </c>
       <c r="Y267" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z267" s="3" t="n">
         <v>-0</v>
@@ -31391,7 +31391,7 @@
         <v>0</v>
       </c>
       <c r="Z273" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA273" s="3" t="n">
         <v>1</v>
@@ -31591,7 +31591,7 @@
         <v>0</v>
       </c>
       <c r="Z275" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA275" s="3" t="n">
         <v>1</v>
@@ -31888,7 +31888,7 @@
         <v>0.001032</v>
       </c>
       <c r="Y278" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z278" s="3" t="n">
         <v>-0</v>
@@ -31991,7 +31991,7 @@
         <v>-0</v>
       </c>
       <c r="Z279" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA279" s="3" t="n">
         <v>0</v>
@@ -32191,7 +32191,7 @@
         <v>0</v>
       </c>
       <c r="Z281" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA281" s="3" t="n">
         <v>0</v>
@@ -32288,10 +32288,10 @@
         <v>0.0009479999999999999</v>
       </c>
       <c r="Y282" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z282" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA282" s="3" t="n">
         <v>0</v>
@@ -32588,7 +32588,7 @@
         <v>0.00143</v>
       </c>
       <c r="Y285" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z285" s="3" t="n">
         <v>-0</v>
@@ -32891,7 +32891,7 @@
         <v>0</v>
       </c>
       <c r="Z288" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA288" s="3" t="n">
         <v>1</v>
@@ -33088,10 +33088,10 @@
         <v>0.00315</v>
       </c>
       <c r="Y290" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z290" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA290" s="3" t="n">
         <v>0</v>
@@ -33291,7 +33291,7 @@
         <v>-0</v>
       </c>
       <c r="Z292" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA292" s="3" t="n">
         <v>0</v>
@@ -33691,7 +33691,7 @@
         <v>0</v>
       </c>
       <c r="Z296" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA296" s="3" t="n">
         <v>0</v>
@@ -33788,7 +33788,7 @@
         <v>0.000837</v>
       </c>
       <c r="Y297" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z297" s="3" t="n">
         <v>-0</v>
@@ -34288,7 +34288,7 @@
         <v>0.00126</v>
       </c>
       <c r="Y302" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z302" s="3" t="n">
         <v>0</v>
@@ -34788,7 +34788,7 @@
         <v>0.000827</v>
       </c>
       <c r="Y307" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z307" s="3" t="n">
         <v>0</v>
@@ -35388,7 +35388,7 @@
         <v>0.001773</v>
       </c>
       <c r="Y313" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z313" s="3" t="n">
         <v>-0</v>
@@ -35491,7 +35491,7 @@
         <v>0</v>
       </c>
       <c r="Z314" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA314" s="3" t="n">
         <v>0</v>
@@ -35991,7 +35991,7 @@
         <v>0</v>
       </c>
       <c r="Z319" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA319" s="3" t="n">
         <v>3</v>
@@ -36088,10 +36088,10 @@
         <v>0.000803</v>
       </c>
       <c r="Y320" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z320" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA320" s="3" t="n">
         <v>1</v>
@@ -37988,10 +37988,10 @@
         <v>0.001203</v>
       </c>
       <c r="Y339" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z339" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA339" s="3" t="n">
         <v>0</v>
@@ -38588,10 +38588,10 @@
         <v>0.000592</v>
       </c>
       <c r="Y345" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z345" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA345" s="3" t="n">
         <v>0</v>
@@ -39388,7 +39388,7 @@
         <v>0.000518</v>
       </c>
       <c r="Y353" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z353" s="3" t="n">
         <v>0</v>
@@ -39556,10 +39556,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.220335</v>
+        <v>0.11126</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.171702</v>
+        <v>0.130604</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.599035</v>
@@ -39610,10 +39610,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.45149</v>
+        <v>0.418443</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.419798</v>
+        <v>0.390682</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.531073</v>
@@ -39985,10 +39985,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.45149</v>
+        <v>0.418443</v>
       </c>
       <c r="E8" t="n">
-        <v>0.34611</v>
+        <v>0.316891</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40015,10 +40015,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.220335</v>
+        <v>0.11126</v>
       </c>
       <c r="E9" t="n">
-        <v>0.164159</v>
+        <v>0.081349</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40045,10 +40045,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.367122</v>
+        <v>0.351733</v>
       </c>
       <c r="E10" t="n">
-        <v>0.29728</v>
+        <v>0.28563</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40075,10 +40075,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.419798</v>
+        <v>0.390682</v>
       </c>
       <c r="E11" t="n">
-        <v>0.316712</v>
+        <v>0.29207</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40105,10 +40105,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.171702</v>
+        <v>0.130604</v>
       </c>
       <c r="E12" t="n">
-        <v>0.123751</v>
+        <v>0.095369</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40135,10 +40135,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.344363</v>
+        <v>0.359874</v>
       </c>
       <c r="E13" t="n">
-        <v>0.27891</v>
+        <v>0.291959</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>

<commit_message>
chore(epirank): refresh ERA results after zero-degree self-loop fix
- regenerate ERA_result json+xlsx for 原 (309), 原_Germany (317), 改 (305/306), 改_Germany (310) with the self-loop patched CN/CNt
- out.py: compare 改 reverse_seqday vs 改 seqday
- remove EpiRank_原_Germany/修改.md
</commit_message>
<xml_diff>
--- a/EpiRank_原/ERA_result_d_0.95_daytime_0.5_loops_309.xlsx
+++ b/EpiRank_原/ERA_result_d_0.95_daytime_0.5_loops_309.xlsx
@@ -714,10 +714,10 @@
         <v>0.012835</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA2" s="3" t="n">
         <v>9</v>
@@ -1334,7 +1334,7 @@
         <v>0.006652</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="3" t="n">
         <v>0</v>
@@ -1636,10 +1636,10 @@
         <v>0.016941</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z8" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA8" s="3" t="n">
         <v>8</v>
@@ -1787,10 +1787,10 @@
         <v>0.011997</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z9" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA9" s="3" t="n">
         <v>4</v>
@@ -2093,10 +2093,10 @@
         <v>0.009434</v>
       </c>
       <c r="Y11" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z11" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA11" s="3" t="n">
         <v>2</v>
@@ -4268,10 +4268,10 @@
         <v>0.007023</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z26" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA26" s="3" t="n">
         <v>8</v>
@@ -6478,10 +6478,10 @@
         <v>0.004917</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>2</v>
@@ -7438,10 +7438,10 @@
         <v>0.005555</v>
       </c>
       <c r="Y52" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z52" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA52" s="3" t="n">
         <v>2</v>
@@ -8401,7 +8401,7 @@
         <v>0</v>
       </c>
       <c r="Z60" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA60" s="3" t="n">
         <v>6</v>
@@ -8881,7 +8881,7 @@
         <v>0</v>
       </c>
       <c r="Z64" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA64" s="3" t="n">
         <v>35</v>
@@ -9578,10 +9578,10 @@
         <v>0.006096</v>
       </c>
       <c r="Y70" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z70" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA70" s="3" t="n">
         <v>1</v>
@@ -10018,10 +10018,10 @@
         <v>0.002648</v>
       </c>
       <c r="Y74" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z74" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA74" s="3" t="n">
         <v>4</v>
@@ -10241,7 +10241,7 @@
         <v>-0</v>
       </c>
       <c r="Z76" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA76" s="3" t="n">
         <v>0</v>
@@ -10788,10 +10788,10 @@
         <v>0.004355</v>
       </c>
       <c r="Y81" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z81" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA81" s="3" t="n">
         <v>0</v>
@@ -11341,7 +11341,7 @@
         <v>0</v>
       </c>
       <c r="Z86" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA86" s="3" t="n">
         <v>1</v>
@@ -11561,7 +11561,7 @@
         <v>0</v>
       </c>
       <c r="Z88" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA88" s="3" t="n">
         <v>2</v>
@@ -11998,10 +11998,10 @@
         <v>0.003408</v>
       </c>
       <c r="Y92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z92" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA92" s="3" t="n">
         <v>1</v>
@@ -12108,10 +12108,10 @@
         <v>0.003716</v>
       </c>
       <c r="Y93" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z93" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA93" s="3" t="n">
         <v>0</v>
@@ -12218,10 +12218,10 @@
         <v>0.002947</v>
       </c>
       <c r="Y94" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z94" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA94" s="3" t="n">
         <v>3</v>
@@ -12328,10 +12328,10 @@
         <v>0.002268</v>
       </c>
       <c r="Y95" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z95" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA95" s="3" t="n">
         <v>0</v>
@@ -12438,10 +12438,10 @@
         <v>0.003781</v>
       </c>
       <c r="Y96" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z96" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA96" s="3" t="n">
         <v>0</v>
@@ -13318,10 +13318,10 @@
         <v>0.003197</v>
       </c>
       <c r="Y104" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z104" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA104" s="3" t="n">
         <v>1</v>
@@ -13538,10 +13538,10 @@
         <v>0.002715</v>
       </c>
       <c r="Y106" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z106" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA106" s="3" t="n">
         <v>1</v>
@@ -14088,7 +14088,7 @@
         <v>0.001988</v>
       </c>
       <c r="Y111" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z111" s="3" t="n">
         <v>-0</v>
@@ -14308,10 +14308,10 @@
         <v>0.002806</v>
       </c>
       <c r="Y113" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z113" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA113" s="3" t="n">
         <v>0</v>
@@ -14748,10 +14748,10 @@
         <v>0.002833</v>
       </c>
       <c r="Y117" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z117" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA117" s="3" t="n">
         <v>1</v>
@@ -15521,7 +15521,7 @@
         <v>0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>0</v>
@@ -15628,10 +15628,10 @@
         <v>0.002787</v>
       </c>
       <c r="Y125" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>2</v>
@@ -15741,7 +15741,7 @@
         <v>0</v>
       </c>
       <c r="Z126" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA126" s="3" t="n">
         <v>0</v>
@@ -16068,10 +16068,10 @@
         <v>0.002014</v>
       </c>
       <c r="Y129" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z129" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA129" s="3" t="n">
         <v>3</v>
@@ -16178,10 +16178,10 @@
         <v>0.002381</v>
       </c>
       <c r="Y130" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z130" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA130" s="3" t="n">
         <v>2</v>
@@ -16398,10 +16398,10 @@
         <v>0.002147</v>
       </c>
       <c r="Y132" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z132" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA132" s="3" t="n">
         <v>1</v>
@@ -16838,10 +16838,10 @@
         <v>0.002116</v>
       </c>
       <c r="Y136" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z136" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA136" s="3" t="n">
         <v>0</v>
@@ -17061,7 +17061,7 @@
         <v>0</v>
       </c>
       <c r="Z138" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA138" s="3" t="n">
         <v>2</v>
@@ -17168,10 +17168,10 @@
         <v>0.002578</v>
       </c>
       <c r="Y139" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z139" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA139" s="3" t="n">
         <v>0</v>
@@ -17391,7 +17391,7 @@
         <v>0</v>
       </c>
       <c r="Z141" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA141" s="3" t="n">
         <v>1</v>
@@ -17498,10 +17498,10 @@
         <v>0.002604</v>
       </c>
       <c r="Y142" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z142" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA142" s="3" t="n">
         <v>7</v>
@@ -17938,10 +17938,10 @@
         <v>0.00181</v>
       </c>
       <c r="Y146" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z146" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA146" s="3" t="n">
         <v>1</v>
@@ -18488,7 +18488,7 @@
         <v>0.002174</v>
       </c>
       <c r="Y151" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z151" s="3" t="n">
         <v>0</v>
@@ -18708,10 +18708,10 @@
         <v>0.001664</v>
       </c>
       <c r="Y153" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z153" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>0</v>
@@ -18818,10 +18818,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y154" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z154" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA154" s="3" t="n">
         <v>0</v>
@@ -19258,10 +19258,10 @@
         <v>0.003403</v>
       </c>
       <c r="Y158" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>0</v>
@@ -19481,7 +19481,7 @@
         <v>-0</v>
       </c>
       <c r="Z160" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA160" s="3" t="n">
         <v>1</v>
@@ -20248,10 +20248,10 @@
         <v>0.002432</v>
       </c>
       <c r="Y167" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z167" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA167" s="3" t="n">
         <v>1</v>
@@ -20908,10 +20908,10 @@
         <v>0.003364</v>
       </c>
       <c r="Y173" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z173" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA173" s="3" t="n">
         <v>0</v>
@@ -21018,10 +21018,10 @@
         <v>0.002818</v>
       </c>
       <c r="Y174" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z174" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA174" s="3" t="n">
         <v>0</v>
@@ -21128,7 +21128,7 @@
         <v>0.001797</v>
       </c>
       <c r="Y175" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z175" s="3" t="n">
         <v>0</v>
@@ -21461,7 +21461,7 @@
         <v>0</v>
       </c>
       <c r="Z178" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA178" s="3" t="n">
         <v>2</v>
@@ -21678,10 +21678,10 @@
         <v>0.001235</v>
       </c>
       <c r="Y180" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z180" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA180" s="3" t="n">
         <v>1</v>
@@ -21788,7 +21788,7 @@
         <v>0.002087</v>
       </c>
       <c r="Y181" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z181" s="3" t="n">
         <v>-0</v>
@@ -22118,7 +22118,7 @@
         <v>0.002161</v>
       </c>
       <c r="Y184" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z184" s="3" t="n">
         <v>-0</v>
@@ -22341,7 +22341,7 @@
         <v>-0</v>
       </c>
       <c r="Z186" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA186" s="3" t="n">
         <v>1</v>
@@ -22448,10 +22448,10 @@
         <v>0.002618</v>
       </c>
       <c r="Y187" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z187" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA187" s="3" t="n">
         <v>0</v>
@@ -22558,10 +22558,10 @@
         <v>0.001669</v>
       </c>
       <c r="Y188" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z188" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA188" s="3" t="n">
         <v>0</v>
@@ -22778,7 +22778,7 @@
         <v>0.00302</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z190" s="3" t="n">
         <v>0</v>
@@ -23001,7 +23001,7 @@
         <v>-0</v>
       </c>
       <c r="Z192" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA192" s="3" t="n">
         <v>0</v>
@@ -23328,10 +23328,10 @@
         <v>0.001901</v>
       </c>
       <c r="Y195" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z195" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA195" s="3" t="n">
         <v>0</v>
@@ -23661,7 +23661,7 @@
         <v>-0</v>
       </c>
       <c r="Z198" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA198" s="3" t="n">
         <v>0</v>
@@ -23988,7 +23988,7 @@
         <v>0.001259</v>
       </c>
       <c r="Y201" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z201" s="3" t="n">
         <v>-0</v>
@@ -24318,7 +24318,7 @@
         <v>0.002004</v>
       </c>
       <c r="Y204" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z204" s="3" t="n">
         <v>0</v>
@@ -24538,7 +24538,7 @@
         <v>0.001782</v>
       </c>
       <c r="Y206" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z206" s="3" t="n">
         <v>-0</v>
@@ -24761,7 +24761,7 @@
         <v>0</v>
       </c>
       <c r="Z208" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA208" s="3" t="n">
         <v>1</v>
@@ -24978,10 +24978,10 @@
         <v>0.001245</v>
       </c>
       <c r="Y210" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>0</v>
@@ -25088,7 +25088,7 @@
         <v>0.001081</v>
       </c>
       <c r="Y211" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z211" s="3" t="n">
         <v>-0</v>
@@ -25638,10 +25638,10 @@
         <v>0.0008140000000000001</v>
       </c>
       <c r="Y216" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z216" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA216" s="3" t="n">
         <v>0</v>
@@ -25748,10 +25748,10 @@
         <v>0.000905</v>
       </c>
       <c r="Y217" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z217" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA217" s="3" t="n">
         <v>0</v>
@@ -26078,7 +26078,7 @@
         <v>0.001943</v>
       </c>
       <c r="Y220" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z220" s="3" t="n">
         <v>-0</v>
@@ -26391,7 +26391,7 @@
         <v>-0</v>
       </c>
       <c r="Z223" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA223" s="3" t="n">
         <v>6</v>
@@ -26588,10 +26588,10 @@
         <v>0.00135</v>
       </c>
       <c r="Y225" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z225" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA225" s="3" t="n">
         <v>0</v>
@@ -26788,7 +26788,7 @@
         <v>0.001152</v>
       </c>
       <c r="Y227" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z227" s="3" t="n">
         <v>-0</v>
@@ -26988,10 +26988,10 @@
         <v>0.00125</v>
       </c>
       <c r="Y229" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z229" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA229" s="3" t="n">
         <v>0</v>
@@ -27291,7 +27291,7 @@
         <v>0</v>
       </c>
       <c r="Z232" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA232" s="3" t="n">
         <v>0</v>
@@ -27588,10 +27588,10 @@
         <v>0.001309</v>
       </c>
       <c r="Y235" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z235" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA235" s="3" t="n">
         <v>0</v>
@@ -27688,7 +27688,7 @@
         <v>0.001592</v>
       </c>
       <c r="Y236" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z236" s="3" t="n">
         <v>-0</v>
@@ -28388,10 +28388,10 @@
         <v>0.001248</v>
       </c>
       <c r="Y243" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z243" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA243" s="3" t="n">
         <v>0</v>
@@ -28591,7 +28591,7 @@
         <v>0</v>
       </c>
       <c r="Z245" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA245" s="3" t="n">
         <v>1</v>
@@ -28688,10 +28688,10 @@
         <v>0.002084</v>
       </c>
       <c r="Y246" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z246" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA246" s="3" t="n">
         <v>2</v>
@@ -28788,10 +28788,10 @@
         <v>0.001352</v>
       </c>
       <c r="Y247" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z247" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z247" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA247" s="3" t="n">
         <v>0</v>
@@ -28891,7 +28891,7 @@
         <v>0</v>
       </c>
       <c r="Z248" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA248" s="3" t="n">
         <v>0</v>
@@ -28988,10 +28988,10 @@
         <v>0.001148</v>
       </c>
       <c r="Y249" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z249" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA249" s="3" t="n">
         <v>0</v>
@@ -29088,10 +29088,10 @@
         <v>0.001877</v>
       </c>
       <c r="Y250" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z250" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA250" s="3" t="n">
         <v>0</v>
@@ -29388,7 +29388,7 @@
         <v>0.001506</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z253" s="3" t="n">
         <v>-0</v>
@@ -29488,7 +29488,7 @@
         <v>0.001296</v>
       </c>
       <c r="Y254" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z254" s="3" t="n">
         <v>0</v>
@@ -29691,7 +29691,7 @@
         <v>-0</v>
       </c>
       <c r="Z256" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA256" s="3" t="n">
         <v>0</v>
@@ -29891,7 +29891,7 @@
         <v>0</v>
       </c>
       <c r="Z258" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA258" s="3" t="n">
         <v>2</v>
@@ -30088,10 +30088,10 @@
         <v>0.000867</v>
       </c>
       <c r="Y260" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z260" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA260" s="3" t="n">
         <v>0</v>
@@ -30288,10 +30288,10 @@
         <v>0.000785</v>
       </c>
       <c r="Y262" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z262" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA262" s="3" t="n">
         <v>0</v>
@@ -30788,10 +30788,10 @@
         <v>0.001386</v>
       </c>
       <c r="Y267" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z267" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA267" s="3" t="n">
         <v>0</v>
@@ -32191,7 +32191,7 @@
         <v>0</v>
       </c>
       <c r="Z281" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA281" s="3" t="n">
         <v>0</v>
@@ -32291,7 +32291,7 @@
         <v>-0</v>
       </c>
       <c r="Z282" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA282" s="3" t="n">
         <v>0</v>
@@ -32591,7 +32591,7 @@
         <v>-0</v>
       </c>
       <c r="Z285" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA285" s="3" t="n">
         <v>0</v>
@@ -32688,10 +32688,10 @@
         <v>0.00209</v>
       </c>
       <c r="Y286" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>1</v>
@@ -33288,10 +33288,10 @@
         <v>0.001184</v>
       </c>
       <c r="Y292" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z292" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA292" s="3" t="n">
         <v>0</v>
@@ -33588,10 +33588,10 @@
         <v>0.001378</v>
       </c>
       <c r="Y295" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z295" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA295" s="3" t="n">
         <v>2</v>
@@ -34091,7 +34091,7 @@
         <v>0</v>
       </c>
       <c r="Z300" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA300" s="3" t="n">
         <v>9</v>
@@ -34291,7 +34291,7 @@
         <v>-0</v>
       </c>
       <c r="Z302" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA302" s="3" t="n">
         <v>0</v>
@@ -34491,7 +34491,7 @@
         <v>0</v>
       </c>
       <c r="Z304" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA304" s="3" t="n">
         <v>0</v>
@@ -34688,10 +34688,10 @@
         <v>0.001202</v>
       </c>
       <c r="Y306" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z306" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA306" s="3" t="n">
         <v>0</v>
@@ -34791,7 +34791,7 @@
         <v>-0</v>
       </c>
       <c r="Z307" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA307" s="3" t="n">
         <v>0</v>
@@ -34888,10 +34888,10 @@
         <v>0.001097</v>
       </c>
       <c r="Y308" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z308" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA308" s="3" t="n">
         <v>0</v>
@@ -34988,10 +34988,10 @@
         <v>0.000803</v>
       </c>
       <c r="Y309" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z309" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA309" s="3" t="n">
         <v>0</v>
@@ -35188,7 +35188,7 @@
         <v>0.001123</v>
       </c>
       <c r="Y311" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z311" s="3" t="n">
         <v>0</v>
@@ -35391,7 +35391,7 @@
         <v>-0</v>
       </c>
       <c r="Z313" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA313" s="3" t="n">
         <v>1</v>
@@ -35791,7 +35791,7 @@
         <v>0</v>
       </c>
       <c r="Z317" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA317" s="3" t="n">
         <v>0</v>
@@ -36091,7 +36091,7 @@
         <v>-0</v>
       </c>
       <c r="Z320" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA320" s="3" t="n">
         <v>1</v>
@@ -36488,10 +36488,10 @@
         <v>0.00087</v>
       </c>
       <c r="Y324" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z324" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA324" s="3" t="n">
         <v>0</v>
@@ -37888,10 +37888,10 @@
         <v>0.00122</v>
       </c>
       <c r="Y338" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z338" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA338" s="3" t="n">
         <v>0</v>
@@ -37991,7 +37991,7 @@
         <v>-0</v>
       </c>
       <c r="Z339" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA339" s="3" t="n">
         <v>0</v>
@@ -38488,7 +38488,7 @@
         <v>0.000561</v>
       </c>
       <c r="Y344" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z344" s="3" t="n">
         <v>0</v>
@@ -38591,7 +38591,7 @@
         <v>-0</v>
       </c>
       <c r="Z345" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA345" s="3" t="n">
         <v>0</v>
@@ -39391,7 +39391,7 @@
         <v>-0</v>
       </c>
       <c r="Z353" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA353" s="3" t="n">
         <v>0</v>
@@ -39556,10 +39556,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.11126</v>
+        <v>0.047472</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.130604</v>
+        <v>0.078362</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.599035</v>
@@ -39610,10 +39610,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.418443</v>
+        <v>0.380211</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.390682</v>
+        <v>0.358513</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.531073</v>
@@ -39985,10 +39985,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.418443</v>
+        <v>0.380211</v>
       </c>
       <c r="E8" t="n">
-        <v>0.316891</v>
+        <v>0.28599</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40015,10 +40015,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.11126</v>
+        <v>0.047472</v>
       </c>
       <c r="E9" t="n">
-        <v>0.081349</v>
+        <v>0.034619</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40045,10 +40045,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.351733</v>
+        <v>0.323194</v>
       </c>
       <c r="E10" t="n">
-        <v>0.28563</v>
+        <v>0.261212</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40075,10 +40075,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.390682</v>
+        <v>0.358513</v>
       </c>
       <c r="E11" t="n">
-        <v>0.29207</v>
+        <v>0.265283</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40105,10 +40105,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.130604</v>
+        <v>0.078362</v>
       </c>
       <c r="E12" t="n">
-        <v>0.095369</v>
+        <v>0.05898</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40135,10 +40135,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.359874</v>
+        <v>0.310017</v>
       </c>
       <c r="E13" t="n">
-        <v>0.291959</v>
+        <v>0.249899</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>

<commit_message>
feat(epirank): add SARS panels and rework core-count tables in all GUI variants
- Tab 5 Frequency Distribution: widen to (18,10) and 2x3 grid, add SARS freq + in/out ratio panels (c)/(f)
- Tab 7 EpiRank vs Disease: widen to (18,6) and 1x3 grid, add SARS comparison panel (c)
- Table 1: add Flu/EV/SARS rows and an 'all core (I+II+III)' row, keep NC row; fixed row heights
- rework core-overlap table into a single compact widget
- out.py: compare 原 (ERA_result_d_) vs 改 (ERA_result_seqday_d_)
- refresh ERA_result json+xlsx (原 309, 原_Germany 317, 改 305, 改_Germany 310)
</commit_message>
<xml_diff>
--- a/EpiRank_原/ERA_result_d_0.95_daytime_0.5_loops_309.xlsx
+++ b/EpiRank_原/ERA_result_d_0.95_daytime_0.5_loops_309.xlsx
@@ -714,10 +714,10 @@
         <v>0.012835</v>
       </c>
       <c r="Y2" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z2" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA2" s="3" t="n">
         <v>9</v>
@@ -1179,10 +1179,10 @@
         <v>0.01205</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="3" t="n">
         <v>11</v>
@@ -1787,10 +1787,10 @@
         <v>0.011997</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA9" s="3" t="n">
         <v>4</v>
@@ -2093,10 +2093,10 @@
         <v>0.009434</v>
       </c>
       <c r="Y11" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="3" t="n">
         <v>2</v>
@@ -2708,10 +2708,10 @@
         <v>0.004698</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z15" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA15" s="3" t="n">
         <v>4</v>
@@ -3008,10 +3008,10 @@
         <v>0.008274999999999999</v>
       </c>
       <c r="Y17" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA17" s="3" t="n">
         <v>4</v>
@@ -3158,10 +3158,10 @@
         <v>0.008586</v>
       </c>
       <c r="Y18" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA18" s="3" t="n">
         <v>3</v>
@@ -4528,10 +4528,10 @@
         <v>0.01038</v>
       </c>
       <c r="Y28" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA28" s="3" t="n">
         <v>0</v>
@@ -4658,10 +4658,10 @@
         <v>0.009729</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA29" s="3" t="n">
         <v>24</v>
@@ -5038,10 +5038,10 @@
         <v>0.005408</v>
       </c>
       <c r="Y32" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z32" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA32" s="3" t="n">
         <v>7</v>
@@ -5518,10 +5518,10 @@
         <v>0.008265</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA36" s="3" t="n">
         <v>5</v>
@@ -6478,10 +6478,10 @@
         <v>0.004917</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA44" s="3" t="n">
         <v>2</v>
@@ -7438,10 +7438,10 @@
         <v>0.005555</v>
       </c>
       <c r="Y52" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z52" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA52" s="3" t="n">
         <v>2</v>
@@ -8878,10 +8878,10 @@
         <v>0.0015</v>
       </c>
       <c r="Y64" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z64" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA64" s="3" t="n">
         <v>35</v>
@@ -10348,7 +10348,7 @@
         <v>0.002616</v>
       </c>
       <c r="Y77" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z77" s="3" t="n">
         <v>-0</v>
@@ -11338,10 +11338,10 @@
         <v>0.003041</v>
       </c>
       <c r="Y86" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z86" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA86" s="3" t="n">
         <v>1</v>
@@ -12218,10 +12218,10 @@
         <v>0.002947</v>
       </c>
       <c r="Y94" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z94" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA94" s="3" t="n">
         <v>3</v>
@@ -12328,10 +12328,10 @@
         <v>0.002268</v>
       </c>
       <c r="Y95" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z95" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA95" s="3" t="n">
         <v>0</v>
@@ -12658,10 +12658,10 @@
         <v>0.0059</v>
       </c>
       <c r="Y98" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z98" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA98" s="3" t="n">
         <v>0</v>
@@ -12878,10 +12878,10 @@
         <v>0.003369</v>
       </c>
       <c r="Y100" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z100" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA100" s="3" t="n">
         <v>2</v>
@@ -14308,10 +14308,10 @@
         <v>0.002806</v>
       </c>
       <c r="Y113" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z113" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA113" s="3" t="n">
         <v>0</v>
@@ -14748,10 +14748,10 @@
         <v>0.002833</v>
       </c>
       <c r="Y117" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z117" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA117" s="3" t="n">
         <v>1</v>
@@ -14858,10 +14858,10 @@
         <v>0.002496</v>
       </c>
       <c r="Y118" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z118" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA118" s="3" t="n">
         <v>1</v>
@@ -15408,10 +15408,10 @@
         <v>0.002594</v>
       </c>
       <c r="Y123" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z123" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA123" s="3" t="n">
         <v>0</v>
@@ -15521,7 +15521,7 @@
         <v>0</v>
       </c>
       <c r="Z124" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA124" s="3" t="n">
         <v>0</v>
@@ -15628,10 +15628,10 @@
         <v>0.002787</v>
       </c>
       <c r="Y125" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z125" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA125" s="3" t="n">
         <v>2</v>
@@ -15741,7 +15741,7 @@
         <v>0</v>
       </c>
       <c r="Z126" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA126" s="3" t="n">
         <v>0</v>
@@ -15961,7 +15961,7 @@
         <v>0</v>
       </c>
       <c r="Z128" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA128" s="3" t="n">
         <v>1</v>
@@ -16068,10 +16068,10 @@
         <v>0.002014</v>
       </c>
       <c r="Y129" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z129" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA129" s="3" t="n">
         <v>3</v>
@@ -16398,10 +16398,10 @@
         <v>0.002147</v>
       </c>
       <c r="Y132" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z132" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA132" s="3" t="n">
         <v>1</v>
@@ -16508,10 +16508,10 @@
         <v>0.003344</v>
       </c>
       <c r="Y133" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z133" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA133" s="3" t="n">
         <v>3</v>
@@ -16728,10 +16728,10 @@
         <v>0.004587</v>
       </c>
       <c r="Y135" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z135" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA135" s="3" t="n">
         <v>0</v>
@@ -17061,7 +17061,7 @@
         <v>0</v>
       </c>
       <c r="Z138" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA138" s="3" t="n">
         <v>2</v>
@@ -17498,7 +17498,7 @@
         <v>0.002604</v>
       </c>
       <c r="Y142" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z142" s="3" t="n">
         <v>0</v>
@@ -17718,10 +17718,10 @@
         <v>0.005244</v>
       </c>
       <c r="Y144" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z144" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA144" s="3" t="n">
         <v>2</v>
@@ -17828,10 +17828,10 @@
         <v>0.001714</v>
       </c>
       <c r="Y145" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z145" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA145" s="3" t="n">
         <v>2</v>
@@ -17938,10 +17938,10 @@
         <v>0.00181</v>
       </c>
       <c r="Y146" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z146" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA146" s="3" t="n">
         <v>1</v>
@@ -18491,7 +18491,7 @@
         <v>-0</v>
       </c>
       <c r="Z151" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA151" s="3" t="n">
         <v>1</v>
@@ -18708,10 +18708,10 @@
         <v>0.001664</v>
       </c>
       <c r="Y153" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z153" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z153" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA153" s="3" t="n">
         <v>0</v>
@@ -18818,10 +18818,10 @@
         <v>0.001295</v>
       </c>
       <c r="Y154" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z154" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA154" s="3" t="n">
         <v>0</v>
@@ -19258,10 +19258,10 @@
         <v>0.003403</v>
       </c>
       <c r="Y158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z158" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA158" s="3" t="n">
         <v>0</v>
@@ -19368,10 +19368,10 @@
         <v>0.002542</v>
       </c>
       <c r="Y159" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z159" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA159" s="3" t="n">
         <v>1</v>
@@ -19478,7 +19478,7 @@
         <v>0.004473</v>
       </c>
       <c r="Y160" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z160" s="3" t="n">
         <v>0</v>
@@ -19808,10 +19808,10 @@
         <v>0.002964</v>
       </c>
       <c r="Y163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z163" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA163" s="3" t="n">
         <v>3</v>
@@ -20028,10 +20028,10 @@
         <v>0.002813</v>
       </c>
       <c r="Y165" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z165" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA165" s="3" t="n">
         <v>1</v>
@@ -20138,7 +20138,7 @@
         <v>0.001963</v>
       </c>
       <c r="Y166" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z166" s="3" t="n">
         <v>-0</v>
@@ -20251,7 +20251,7 @@
         <v>-0</v>
       </c>
       <c r="Z167" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA167" s="3" t="n">
         <v>1</v>
@@ -21018,7 +21018,7 @@
         <v>0.002818</v>
       </c>
       <c r="Y174" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z174" s="3" t="n">
         <v>-0</v>
@@ -21131,7 +21131,7 @@
         <v>-0</v>
       </c>
       <c r="Z175" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA175" s="3" t="n">
         <v>0</v>
@@ -21241,7 +21241,7 @@
         <v>0</v>
       </c>
       <c r="Z176" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA176" s="3" t="n">
         <v>1</v>
@@ -21458,10 +21458,10 @@
         <v>0.001262</v>
       </c>
       <c r="Y178" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z178" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA178" s="3" t="n">
         <v>2</v>
@@ -21788,7 +21788,7 @@
         <v>0.002087</v>
       </c>
       <c r="Y181" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z181" s="3" t="n">
         <v>-0</v>
@@ -21901,7 +21901,7 @@
         <v>0</v>
       </c>
       <c r="Z182" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA182" s="3" t="n">
         <v>0</v>
@@ -22118,10 +22118,10 @@
         <v>0.002161</v>
       </c>
       <c r="Y184" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z184" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA184" s="3" t="n">
         <v>0</v>
@@ -22341,7 +22341,7 @@
         <v>-0</v>
       </c>
       <c r="Z186" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA186" s="3" t="n">
         <v>1</v>
@@ -22668,7 +22668,7 @@
         <v>0.0009700000000000001</v>
       </c>
       <c r="Y189" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z189" s="3" t="n">
         <v>-0</v>
@@ -22778,7 +22778,7 @@
         <v>0.00302</v>
       </c>
       <c r="Y190" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z190" s="3" t="n">
         <v>0</v>
@@ -22888,7 +22888,7 @@
         <v>0.001708</v>
       </c>
       <c r="Y191" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z191" s="3" t="n">
         <v>-0</v>
@@ -22998,10 +22998,10 @@
         <v>0.002238</v>
       </c>
       <c r="Y192" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z192" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA192" s="3" t="n">
         <v>0</v>
@@ -23328,10 +23328,10 @@
         <v>0.001901</v>
       </c>
       <c r="Y195" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z195" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA195" s="3" t="n">
         <v>0</v>
@@ -23438,10 +23438,10 @@
         <v>0.001326</v>
       </c>
       <c r="Y196" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z196" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA196" s="3" t="n">
         <v>0</v>
@@ -23658,7 +23658,7 @@
         <v>0.001192</v>
       </c>
       <c r="Y198" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z198" s="3" t="n">
         <v>0</v>
@@ -23768,7 +23768,7 @@
         <v>0.00185</v>
       </c>
       <c r="Y199" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z199" s="3" t="n">
         <v>0</v>
@@ -23878,10 +23878,10 @@
         <v>0.001686</v>
       </c>
       <c r="Y200" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z200" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA200" s="3" t="n">
         <v>1</v>
@@ -23988,10 +23988,10 @@
         <v>0.001259</v>
       </c>
       <c r="Y201" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z201" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA201" s="3" t="n">
         <v>1</v>
@@ -24761,7 +24761,7 @@
         <v>0</v>
       </c>
       <c r="Z208" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA208" s="3" t="n">
         <v>1</v>
@@ -24978,10 +24978,10 @@
         <v>0.001245</v>
       </c>
       <c r="Y210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z210" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA210" s="3" t="n">
         <v>0</v>
@@ -25091,7 +25091,7 @@
         <v>0</v>
       </c>
       <c r="Z211" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA211" s="3" t="n">
         <v>3</v>
@@ -25308,7 +25308,7 @@
         <v>0.001495</v>
       </c>
       <c r="Y213" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z213" s="3" t="n">
         <v>-0</v>
@@ -25528,10 +25528,10 @@
         <v>0.002059</v>
       </c>
       <c r="Y215" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z215" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA215" s="3" t="n">
         <v>0</v>
@@ -25748,7 +25748,7 @@
         <v>0.000905</v>
       </c>
       <c r="Y217" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z217" s="3" t="n">
         <v>-0</v>
@@ -25858,10 +25858,10 @@
         <v>0.001577</v>
       </c>
       <c r="Y218" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z218" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA218" s="3" t="n">
         <v>0</v>
@@ -26078,7 +26078,7 @@
         <v>0.001943</v>
       </c>
       <c r="Y220" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z220" s="3" t="n">
         <v>-0</v>
@@ -26388,10 +26388,10 @@
         <v>0.001119</v>
       </c>
       <c r="Y223" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z223" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA223" s="3" t="n">
         <v>6</v>
@@ -26588,10 +26588,10 @@
         <v>0.00135</v>
       </c>
       <c r="Y225" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z225" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA225" s="3" t="n">
         <v>0</v>
@@ -26688,7 +26688,7 @@
         <v>0.001255</v>
       </c>
       <c r="Y226" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z226" s="3" t="n">
         <v>0</v>
@@ -26988,10 +26988,10 @@
         <v>0.00125</v>
       </c>
       <c r="Y229" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z229" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA229" s="3" t="n">
         <v>0</v>
@@ -27188,10 +27188,10 @@
         <v>0.001509</v>
       </c>
       <c r="Y231" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z231" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA231" s="3" t="n">
         <v>0</v>
@@ -27291,7 +27291,7 @@
         <v>0</v>
       </c>
       <c r="Z232" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA232" s="3" t="n">
         <v>0</v>
@@ -27488,10 +27488,10 @@
         <v>0.001</v>
       </c>
       <c r="Y234" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z234" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA234" s="3" t="n">
         <v>1</v>
@@ -27588,10 +27588,10 @@
         <v>0.001309</v>
       </c>
       <c r="Y235" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z235" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA235" s="3" t="n">
         <v>0</v>
@@ -27788,10 +27788,10 @@
         <v>0.00164</v>
       </c>
       <c r="Y237" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z237" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA237" s="3" t="n">
         <v>0</v>
@@ -27991,7 +27991,7 @@
         <v>0</v>
       </c>
       <c r="Z239" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA239" s="3" t="n">
         <v>2</v>
@@ -28388,7 +28388,7 @@
         <v>0.001248</v>
       </c>
       <c r="Y243" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z243" s="3" t="n">
         <v>-0</v>
@@ -28591,7 +28591,7 @@
         <v>0</v>
       </c>
       <c r="Z245" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA245" s="3" t="n">
         <v>1</v>
@@ -28688,10 +28688,10 @@
         <v>0.002084</v>
       </c>
       <c r="Y246" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z246" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA246" s="3" t="n">
         <v>2</v>
@@ -28788,7 +28788,7 @@
         <v>0.001352</v>
       </c>
       <c r="Y247" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z247" s="3" t="n">
         <v>-0</v>
@@ -28891,7 +28891,7 @@
         <v>0</v>
       </c>
       <c r="Z248" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA248" s="3" t="n">
         <v>0</v>
@@ -28991,7 +28991,7 @@
         <v>-0</v>
       </c>
       <c r="Z249" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA249" s="3" t="n">
         <v>0</v>
@@ -29088,10 +29088,10 @@
         <v>0.001877</v>
       </c>
       <c r="Y250" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z250" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA250" s="3" t="n">
         <v>0</v>
@@ -29188,10 +29188,10 @@
         <v>0.001237</v>
       </c>
       <c r="Y251" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z251" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA251" s="3" t="n">
         <v>5</v>
@@ -29388,10 +29388,10 @@
         <v>0.001506</v>
       </c>
       <c r="Y253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z253" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA253" s="3" t="n">
         <v>2</v>
@@ -29491,7 +29491,7 @@
         <v>-0</v>
       </c>
       <c r="Z254" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA254" s="3" t="n">
         <v>1</v>
@@ -29688,10 +29688,10 @@
         <v>0.000995</v>
       </c>
       <c r="Y256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z256" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA256" s="3" t="n">
         <v>0</v>
@@ -29988,7 +29988,7 @@
         <v>0.00134</v>
       </c>
       <c r="Y259" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z259" s="3" t="n">
         <v>0</v>
@@ -30091,7 +30091,7 @@
         <v>-0</v>
       </c>
       <c r="Z260" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA260" s="3" t="n">
         <v>0</v>
@@ -30188,10 +30188,10 @@
         <v>0.001556</v>
       </c>
       <c r="Y261" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z261" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA261" s="3" t="n">
         <v>0</v>
@@ -30291,7 +30291,7 @@
         <v>0</v>
       </c>
       <c r="Z262" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA262" s="3" t="n">
         <v>0</v>
@@ -30588,7 +30588,7 @@
         <v>0.00079</v>
       </c>
       <c r="Y265" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z265" s="3" t="n">
         <v>-0</v>
@@ -30791,7 +30791,7 @@
         <v>-0</v>
       </c>
       <c r="Z267" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA267" s="3" t="n">
         <v>0</v>
@@ -31391,7 +31391,7 @@
         <v>0</v>
       </c>
       <c r="Z273" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA273" s="3" t="n">
         <v>1</v>
@@ -31591,7 +31591,7 @@
         <v>0</v>
       </c>
       <c r="Z275" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA275" s="3" t="n">
         <v>1</v>
@@ -31891,7 +31891,7 @@
         <v>0</v>
       </c>
       <c r="Z278" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA278" s="3" t="n">
         <v>0</v>
@@ -31991,7 +31991,7 @@
         <v>-0</v>
       </c>
       <c r="Z279" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA279" s="3" t="n">
         <v>0</v>
@@ -32188,7 +32188,7 @@
         <v>0.001133</v>
       </c>
       <c r="Y281" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z281" s="3" t="n">
         <v>-0</v>
@@ -32288,10 +32288,10 @@
         <v>0.0009479999999999999</v>
       </c>
       <c r="Y282" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z282" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA282" s="3" t="n">
         <v>0</v>
@@ -32588,7 +32588,7 @@
         <v>0.00143</v>
       </c>
       <c r="Y285" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z285" s="3" t="n">
         <v>0</v>
@@ -32688,10 +32688,10 @@
         <v>0.00209</v>
       </c>
       <c r="Y286" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z286" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA286" s="3" t="n">
         <v>1</v>
@@ -32891,7 +32891,7 @@
         <v>0</v>
       </c>
       <c r="Z288" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA288" s="3" t="n">
         <v>1</v>
@@ -33088,10 +33088,10 @@
         <v>0.00315</v>
       </c>
       <c r="Y290" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z290" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z290" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA290" s="3" t="n">
         <v>0</v>
@@ -33591,7 +33591,7 @@
         <v>-0</v>
       </c>
       <c r="Z295" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA295" s="3" t="n">
         <v>2</v>
@@ -34088,7 +34088,7 @@
         <v>0.001087</v>
       </c>
       <c r="Y300" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z300" s="3" t="n">
         <v>-0</v>
@@ -34288,7 +34288,7 @@
         <v>0.00126</v>
       </c>
       <c r="Y302" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z302" s="3" t="n">
         <v>-0</v>
@@ -34488,10 +34488,10 @@
         <v>0.000908</v>
       </c>
       <c r="Y304" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Z304" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA304" s="3" t="n">
         <v>0</v>
@@ -34688,7 +34688,7 @@
         <v>0.001202</v>
       </c>
       <c r="Y306" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z306" s="3" t="n">
         <v>0</v>
@@ -34888,7 +34888,7 @@
         <v>0.001097</v>
       </c>
       <c r="Y308" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z308" s="3" t="n">
         <v>0</v>
@@ -35188,7 +35188,7 @@
         <v>0.001123</v>
       </c>
       <c r="Y311" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z311" s="3" t="n">
         <v>0</v>
@@ -35388,10 +35388,10 @@
         <v>0.001773</v>
       </c>
       <c r="Y313" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z313" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z313" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA313" s="3" t="n">
         <v>1</v>
@@ -35791,7 +35791,7 @@
         <v>0</v>
       </c>
       <c r="Z317" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA317" s="3" t="n">
         <v>0</v>
@@ -36088,10 +36088,10 @@
         <v>0.000803</v>
       </c>
       <c r="Y320" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z320" s="3" t="n">
         <v>-0</v>
-      </c>
-      <c r="Z320" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="AA320" s="3" t="n">
         <v>1</v>
@@ -36488,10 +36488,10 @@
         <v>0.00087</v>
       </c>
       <c r="Y324" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z324" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA324" s="3" t="n">
         <v>0</v>
@@ -37091,7 +37091,7 @@
         <v>0</v>
       </c>
       <c r="Z330" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA330" s="3" t="n">
         <v>0</v>
@@ -37691,7 +37691,7 @@
         <v>0</v>
       </c>
       <c r="Z336" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA336" s="3" t="n">
         <v>1</v>
@@ -37888,10 +37888,10 @@
         <v>0.00122</v>
       </c>
       <c r="Y338" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z338" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA338" s="3" t="n">
         <v>0</v>
@@ -37988,7 +37988,7 @@
         <v>0.001203</v>
       </c>
       <c r="Y339" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z339" s="3" t="n">
         <v>0</v>
@@ -38191,7 +38191,7 @@
         <v>0</v>
       </c>
       <c r="Z341" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA341" s="3" t="n">
         <v>0</v>
@@ -38488,7 +38488,7 @@
         <v>0.000561</v>
       </c>
       <c r="Y344" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z344" s="3" t="n">
         <v>0</v>
@@ -38588,10 +38588,10 @@
         <v>0.000592</v>
       </c>
       <c r="Y345" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z345" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA345" s="3" t="n">
         <v>0</v>
@@ -39388,10 +39388,10 @@
         <v>0.000518</v>
       </c>
       <c r="Y353" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z353" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA353" s="3" t="n">
         <v>0</v>
@@ -39556,10 +39556,10 @@
         <v>0.529801</v>
       </c>
       <c r="Y356" s="3" t="n">
-        <v>0.047472</v>
+        <v>0.172952</v>
       </c>
       <c r="Z356" s="3" t="n">
-        <v>0.078362</v>
+        <v>0.148901</v>
       </c>
       <c r="AB356" s="3" t="n">
         <v>0.599035</v>
@@ -39610,10 +39610,10 @@
         <v>0.445424</v>
       </c>
       <c r="Y358" s="3" t="n">
-        <v>0.380211</v>
+        <v>0.393498</v>
       </c>
       <c r="Z358" s="3" t="n">
-        <v>0.358513</v>
+        <v>0.382398</v>
       </c>
       <c r="AA358" s="3" t="n">
         <v>0.531073</v>
@@ -39985,10 +39985,10 @@
         <v>0.386474</v>
       </c>
       <c r="D8" t="n">
-        <v>0.380211</v>
+        <v>0.393498</v>
       </c>
       <c r="E8" t="n">
-        <v>0.28599</v>
+        <v>0.302585</v>
       </c>
       <c r="F8" t="n">
         <v>0.2988505747126437</v>
@@ -40015,10 +40015,10 @@
         <v>0.216528</v>
       </c>
       <c r="D9" t="n">
-        <v>0.047472</v>
+        <v>0.172952</v>
       </c>
       <c r="E9" t="n">
-        <v>0.034619</v>
+        <v>0.130073</v>
       </c>
       <c r="F9" t="n">
         <v>0.1641791044776119</v>
@@ -40045,10 +40045,10 @@
         <v>0.41859</v>
       </c>
       <c r="D10" t="n">
-        <v>0.323194</v>
+        <v>0.366272</v>
       </c>
       <c r="E10" t="n">
-        <v>0.261212</v>
+        <v>0.297168</v>
       </c>
       <c r="F10" t="n">
         <v>0.3636363636363636</v>
@@ -40075,10 +40075,10 @@
         <v>0.397421</v>
       </c>
       <c r="D11" t="n">
-        <v>0.358513</v>
+        <v>0.382398</v>
       </c>
       <c r="E11" t="n">
-        <v>0.265283</v>
+        <v>0.286491</v>
       </c>
       <c r="F11" t="n">
         <v>0.3333333333333333</v>
@@ -40105,10 +40105,10 @@
         <v>0.219019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.078362</v>
+        <v>0.148901</v>
       </c>
       <c r="E12" t="n">
-        <v>0.05898</v>
+        <v>0.108838</v>
       </c>
       <c r="F12" t="n">
         <v>0.1716417910447761</v>
@@ -40135,10 +40135,10 @@
         <v>0.43754</v>
       </c>
       <c r="D13" t="n">
-        <v>0.310017</v>
+        <v>0.365738</v>
       </c>
       <c r="E13" t="n">
-        <v>0.249899</v>
+        <v>0.296888</v>
       </c>
       <c r="F13" t="n">
         <v>0.3939393939393939</v>

</xml_diff>